<commit_message>
Fix extraction of european_100000pop.csv
</commit_message>
<xml_diff>
--- a/cities/european_100000pop_comments.xlsx
+++ b/cities/european_100000pop_comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianapessoa/Desktop/dataexport/cities/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F1ECF2-85F4-C640-8E86-E81EA2A5A07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E339698-8143-0C45-AF32-F184CE666376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-3620" yWindow="-28200" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2461" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2462" uniqueCount="571">
   <si>
     <t>name_en</t>
   </si>
@@ -6269,7 +6269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>234</v>
       </c>
@@ -6288,9 +6288,11 @@
       <c r="F169">
         <v>140730</v>
       </c>
-      <c r="G169"/>
+      <c r="G169" s="3" t="s">
+        <v>557</v>
+      </c>
       <c r="H169">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>